<commit_message>
Il y a maintenant 10 articles pour ma veille ainsi l'ajout de la consultation des sources
</commit_message>
<xml_diff>
--- a/Tableau-de-synthèse/8 - BTS SIO - Annexe 8-1 - Tableau de synthèse - Epreuve E4 - BTS SIO 2024.xlsx
+++ b/Tableau-de-synthèse/8 - BTS SIO - Annexe 8-1 - Tableau de synthèse - Epreuve E4 - BTS SIO 2024.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minei\Documents\portfolio_cybersecurite_elegant\Tableau-de-synthèse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5E99703-9532-4643-B98E-C476BD297780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA94397-9C68-4990-A280-A9477C4C2D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -173,6 +173,15 @@
   <si>
     <t>N° candidat : 02541488301</t>
   </si>
+  <si>
+    <t xml:space="preserve">Projet IMMOSYNC </t>
+  </si>
+  <si>
+    <t>Stage Wordpress : refonte du site lifetag.fr</t>
+  </si>
+  <si>
+    <t>05/01/2026 au 20/02/2026</t>
+  </si>
 </sst>
 </file>
 
@@ -741,38 +750,14 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -805,6 +790,30 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1987,6 +1996,721 @@
             <a:xfrm>
               <a:off x="11999870" y="13916488"/>
               <a:ext cx="341660" cy="239040"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>282406</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>167105</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1035526</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>15729</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="4" name="Encre 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6066FCB8-6C16-310B-61D4-9D5C6BE67FE7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7724160" y="8578070"/>
+            <a:ext cx="753120" cy="361080"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="4" name="Encre 3">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6066FCB8-6C16-310B-61D4-9D5C6BE67FE7}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId38"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7715160" y="8569079"/>
+              <a:ext cx="770760" cy="378702"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>325745</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>111305</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>880505</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>407945</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="9" name="Encre 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{423461F6-6C17-9BB9-81C2-C11CB5F16677}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="9070920" y="8522270"/>
+            <a:ext cx="554760" cy="296640"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="9" name="Encre 8">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{423461F6-6C17-9BB9-81C2-C11CB5F16677}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId40"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="9062280" y="8513630"/>
+              <a:ext cx="572400" cy="314280"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>290022</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>133279</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>913542</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>21863</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId41">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="13" name="Encre 12">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A5C44CF-0DD1-664F-4294-BBE2F183524A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="11642040" y="8544244"/>
+            <a:ext cx="623520" cy="401040"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="13" name="Encre 12">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A5C44CF-0DD1-664F-4294-BBE2F183524A}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId42"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="11633400" y="8535604"/>
+              <a:ext cx="641160" cy="418680"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>334441</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>167090</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>891721</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>433130</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="18" name="Encre 17">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC6E4BDB-6049-55C1-58D1-FB3CAD5A7680}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="12989880" y="8578055"/>
+            <a:ext cx="557280" cy="266040"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="18" name="Encre 17">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC6E4BDB-6049-55C1-58D1-FB3CAD5A7680}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId44"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="12980880" y="8569415"/>
+              <a:ext cx="574920" cy="283680"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>356926</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>99883</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>1027606</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>503083</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="22" name="Encre 21">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71F1D628-9F2F-5C98-A661-E1FE4227D6B1}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="7798680" y="17690497"/>
+            <a:ext cx="670680" cy="403200"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="22" name="Encre 21">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71F1D628-9F2F-5C98-A661-E1FE4227D6B1}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId46"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="7790035" y="17681857"/>
+              <a:ext cx="688329" cy="420840"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>150425</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>66737</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>824705</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>424577</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="27" name="Encre 26">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32BF0600-A5B8-2A1A-1ABA-BC74112064FD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="8895600" y="17657351"/>
+            <a:ext cx="674280" cy="357840"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="27" name="Encre 26">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32BF0600-A5B8-2A1A-1ABA-BC74112064FD}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId48"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="8886600" y="17648351"/>
+              <a:ext cx="691920" cy="375480"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>265764</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>167176</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1013844</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>468856</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId49">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="31" name="Encre 30">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AFF1CA3-BACA-6F18-9D48-1BC5B8A809E2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="10314360" y="17757790"/>
+            <a:ext cx="748080" cy="301680"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="31" name="Encre 30">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1AFF1CA3-BACA-6F18-9D48-1BC5B8A809E2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId50"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="10305360" y="17748790"/>
+              <a:ext cx="765720" cy="319320"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>434382</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>111060</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>879702</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>334620</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="33" name="Encre 32">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DAEC1520-4561-DA94-1966-0A9CE6757FB2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="11786400" y="17701674"/>
+            <a:ext cx="445320" cy="223560"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="33" name="Encre 32">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DAEC1520-4561-DA94-1966-0A9CE6757FB2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId52"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="11777760" y="17692674"/>
+              <a:ext cx="462960" cy="241200"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>400902</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>55260</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>824622</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>412020</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="37" name="Encre 36">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{924A2167-2C2B-7A1B-A4A5-DBC7BB0A602C}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="11752920" y="17645874"/>
+            <a:ext cx="423720" cy="356760"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="37" name="Encre 36">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{924A2167-2C2B-7A1B-A4A5-DBC7BB0A602C}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId54"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="11743920" y="17637234"/>
+              <a:ext cx="441360" cy="374400"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>309601</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>189207</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>869041</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>480447</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="41" name="Encre 40">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D420A4CF-6B5A-8879-4232-4955BB062F67}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="12965040" y="17779821"/>
+            <a:ext cx="559440" cy="291240"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="41" name="Encre 40">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D420A4CF-6B5A-8879-4232-4955BB062F67}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId56"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="12956040" y="17771181"/>
+              <a:ext cx="577080" cy="308880"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>434300</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>133864</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>902660</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>475864</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="46" name="Encre 45">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A2D5755-C2A8-AEFB-85F4-A79CBCE70CB8}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="14393160" y="17724478"/>
+            <a:ext cx="468360" cy="342000"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="46" name="Encre 45">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A2D5755-C2A8-AEFB-85F4-A79CBCE70CB8}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId58"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14384160" y="17715478"/>
+              <a:ext cx="486000" cy="359640"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -2269,7 +2993,35 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">899 0 24575,'-18'2'0,"0"0"0,0 2 0,1 0 0,-1 0 0,1 2 0,0 0 0,0 1 0,-16 10 0,-14 11 0,36-19 0,-2-2 0,1 0 0,-21 9 0,19-10 0,1 0 0,0 0 0,1 2 0,-1-1 0,-15 14 0,-53 54 0,32-28 0,13-16 0,-1-2 0,-1-1 0,-46 24 0,74-46 35,-82 51-1435,78-47-5426</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1588.17">0 155 24575,'242'120'0,"-222"-107"0,0 1 0,0 0 0,-2 1 0,0 1 0,29 33 0,-39-41 0,0-1 0,1 0 0,0 0 0,12 6 0,22 16 0,25 24 0,-39-32 0,35 33 0,-63-53 1,-1-1-48,1 0 0,-1 1 0,1-1 0,0 1-1,-1-1 1,1 1 0,-1-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,1-1-1,-1 1 1,0 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0-1-1,0 1 1,0 0 0,0 0 0,0-1 0,0 2 0</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1588.16">0 155 24575,'242'120'0,"-222"-107"0,0 1 0,0 0 0,-2 1 0,0 1 0,29 33 0,-39-41 0,0-1 0,1 0 0,0 0 0,12 6 0,22 16 0,25 24 0,-39-32 0,35 33 0,-63-53 1,-1-1-48,1 0 0,-1 1 0,1-1 0,0 1-1,-1-1 1,1 1 0,-1-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,1-1-1,-1 1 1,0 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0-1-1,0 1 1,0 0 0,0 0 0,0-1 0,0 2 0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink19.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:14:17.811"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1969 216 24575,'-360'111'-289,"10"21"-291,267-100 446,-743 312 121,595-244 164,211-92-276,2 0 0,-1 2 0,-30 21 0,36-20-6701</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1613.33">422 0 24575,'23'1'0,"0"1"0,0 2 0,38 9 0,-43-9 0,482 162 0,-392-126 0,-5 1 0,-41-16 0,75 20 0,-123-41 0,-1 1 0,0 0 0,0 1 0,-1 0 0,21 13 0,-6 1 0,29 27 0,1-5 0,-40-31 0,27 23 0,17 27 0,-33-32 0,2-1 0,47 35 0,16-9-1365,-70-42-5461</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2297,6 +3049,284 @@
     </inkml:brush>
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">0 393 24575,'0'-4'0,"1"0"0,0 0 0,0 0 0,0 0 0,0 1 0,1-1 0,-1 0 0,1 1 0,0-1 0,0 1 0,0 0 0,1-1 0,-1 1 0,4-3 0,3-4 0,2 0 0,16-12 0,-4 5 0,8-6 0,0-2 0,-2 0 0,33-37 0,-24 24 0,-27 29 0,-1-1 0,16-19 0,18-27-1365</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink20.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:14:26.544"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1540 278 24575,'-31'5'0,"-48"13"0,-42 13 0,-37 18 0,-18 11-1438,-5 5 1438,7-2 0,11-8 0,24-7 0,30-12 0,28-7 468,23-8-468,16-8 238,15-5-7697</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2213.43">86 1 24575,'10'0'0,"0"2"0,1-1 0,-1 1 0,0 1 0,0 0 0,0 0 0,-1 1 0,17 8 0,72 50 0,-76-47 0,88 66 0,-65-46 0,1-2 0,55 31 0,-76-50 0,36 28 0,-42-27 0,0-1 0,43 21 0,7 0 0,76 52 0,-134-79 0,0 0 0,13 14 0,-17-15 0,1 0 0,1 0 0,-1 0 0,17 9 0,-16-12 0,11 6 0,0 0 0,0 2 0,25 20 0,-21-11 110,-8-6-479,1-1 1,0 0-1,37 22 0,-32-25-6457</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink21.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:15:07.744"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1732 373 24575,'-26'1'0,"-1"1"0,2 1 0,-1 1 0,-29 9 0,-98 39 0,123-41 0,-734 334 0,420-166 0,266-136 231,49-26-630,0-2 0,-1 0 0,-59 19 0,63-28-6427</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1432.1">246 1 24575,'4'0'0,"1"0"0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,1 0 0,4 4 0,5 5 0,22 20 0,-4-3 0,70 41 0,-62-43 0,52 43 0,94 94 0,-121-106 0,36 28 0,-53-55 0,-33-21 0,-1 0 0,0 1 0,-1 0 0,19 18 0,-7 0 0,-14-15 0,0-1 0,1 0 0,0-1 0,19 14 0,60 44 0,-60-43 0,49 30 0,-39-39 312,-12-6-1989,-12-2-5149</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink22.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:15:26.188"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1547 31 24575,'-31'10'0,"-43"15"0,-45 29 0,-39 15 0,-19 2-1835,-6 5 1835,17-1 0,22-7 0,19-10 0,26-16 593,19-8-593,18-11 303,14-4-303,11-5 0,10 0 0,11-2-7252</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1451.2">0 1 24575,'49'26'0,"59"44"0,-64-41 0,198 149 0,-149-108 0,189 161 0,-264-215 0,5 1-227,-1 0-1,2-1 1,0-1-1,1-2 1,44 18-1,-43-22-6598</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink23.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:19:13.265"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1422 125 24575,'-5'0'0,"1"0"0,-1 1 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-6 4 0,-10 3 0,-727 309 0,551-228 0,112-59 0,56-21 0,-45 21 0,3 4 0,-38 20 0,84-40-1365,2-3-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1166.09">153 1 24575,'23'9'0,"0"1"0,31 18 0,-16-7 0,609 364 0,-45 34 0,-305-193-1365,-272-205-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink24.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:09.892"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1873 247 24575,'-40'9'0,"0"1"0,1 2 0,-38 18 0,42-16 0,-506 206-650,-293 107-576,595-236 2524,236-90-1256,1 0-1,-1 0 1,1 0 0,-1 0 0,1 0-1,-1 1 1,1-1 0,-4 4 0,6-5-38,0 1 0,0-1 1,0 0-1,0 0 0,-1 0 0,1 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 1-1,-1-1 0,1 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,1 1-1,-1-1 0,0 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 0-1,0 1 0,1-1 0,14 6 54,35-2-1423,-23-3-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1863.49">325 0 24575,'8'1'0,"-2"-1"0,1 1 0,0 1 0,0-1 0,0 1 0,0 1 0,-1-1 0,1 1 0,-1 0 0,7 5 0,8 6 0,28 23 0,-45-34 0,188 132 0,-40-33 0,-44-34 0,-70-47 0,37 28 0,152 125 0,-218-167 0,0 0 0,0 1 0,-1 0 0,0 0 0,0 1 0,6 10 0,-10-14 0,-1 0 0,1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,7 4 0,49 22 0,-48-25 0,0 1 0,0 1 0,0 0 0,17 13 0,-6-1-6,48 28-1,-39-27-1345,-17-9-5474</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink25.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:21.810"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">2078 62 24575,'-51'1'0,"0"3"0,0 2 0,-67 17 0,-143 54 0,131-36 0,-366 99 0,391-113 0,59-16 0,-70 25 0,19-1 0,58-23 0,2 2 0,-68 36 0,79-37 0,0-1 0,-51 17 0,-17 6 0,49-15 0,-46 23 0,90-42 25,-1-1-1,1 1 0,0-1 1,0 1-1,0 0 1,0 0-1,0 0 0,0 0 1,0-1-1,0 1 0,0 0 1,0 1-1,-1 0 1,3-2-77,-1 1 0,0-1 0,0 1 1,1-1-1,-1 1 0,0-1 1,0 1-1,1-1 0,-1 0 0,1 1 1,-1-1-1,0 0 0,1 1 1,-1-1-1,1 0 0,-1 1 0,0-1 1,1 0-1,-1 0 0,1 0 1,-1 1-1,1-1 0,-1 0 0,1 0 1,-1 0-1,1 0 0,-1 0 1,1 0-1,-1 0 0,1 0 0,-1 0 1,2 0-1,19 2-6774</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1234.69">437 0 24575,'487'193'-835,"-28"46"100,-233-103 985,-179-103 121,-1 1 0,63 64 1,-100-90-281,0 0 1,16 10 0,-18-15-251,-1 1-1,0 1 1,0-1 0,-1 1-1,1 0 1,-1 0 0,0 1-1,8 11 1,-6-1-6667</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink26.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:32.915"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1237 0 23673,'-1236'620'0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink27.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:35.605"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 1 24371,'1176'990'0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink28.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:54.014"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1553 94 24575,'-308'112'-703,"-389"199"0,530-230 883,-188 101 450,354-181-604,-20 13 348,21-14-371,0 1 0,-1-1 0,1 0 0,0 0 0,0 0 0,0 0 0,-1 1 0,1-1 0,0 0 0,0 0-1,0 1 1,-1-1 0,1 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,-1 1 0,1-1 0,0 0-1,0 0 1,0 1 0,0-1 0,0 0 0,1 1 0,-1-1 0,0 0 0,0 0 0,0 1 0,0-1 0,0 0 0,0 0 0,0 1-1,1-1 1,-1 0 0,0 0 0,0 1 0,0-1 0,0 0 0,1 0 0,-1 1 0,0-1 0,0 0 0,1 0 0,-1 0 0,0 0 0,0 0-1,1 1 1,-1-1 0,0 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0 0,1 0 0,-1 0 0,0 0-1,0 0 1,1 0 0,3 0-154,0 0-1,0 1 0,0-1 0,0-1 1,0 1-1,0-1 0,0 1 1,5-3-1,11-4-6674</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1346.95">130 1 24575,'6'1'0,"0"0"0,0 0 0,0 0 0,0 1 0,-1 0 0,1 1 0,-1-1 0,0 1 0,1 0 0,-1 0 0,-1 1 0,7 5 0,0-2 0,170 129 0,-82-60 0,143 119 0,-190-143 0,-44-42 0,1 0 0,1-1 0,0 1 0,0-2 0,0 1 0,1-2 0,18 11 0,-12-9 26,-1 1 0,-1 0-1,0 1 1,0 1 0,-1 0-1,0 1 1,13 17 0,35 32-1597,-47-50-5255</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink29.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:21:47.723"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1300 62 24575,'-2'0'0,"0"0"0,0 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-3 2 0,-9 5 0,-411 156 0,21-10 0,299-116 0,78-29 0,0 0 0,0 1 0,1 2 0,-25 15 0,-54 35-1365,80-50-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1460.05">0 0 24575,'1'3'0,"0"0"0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,4 3 0,2 5 0,16 15 0,1 0 0,1-2 0,50 36 0,-50-40 0,-6-1 0,0 1 0,-1 0 0,-1 1 0,25 38 0,7 7 0,31 29 0,110 100 0,-156-159 167,36 47 0,-46-51-734,2-1 1,51 45 0,-59-60-6260</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -2796,56 +3826,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+      <c r="D1" s="30"/>
+      <c r="E1" s="30"/>
+      <c r="F1" s="30"/>
+      <c r="G1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="28"/>
+      <c r="H1" s="30"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="29" t="s">
+      <c r="A3" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="30"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="35" t="s">
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="44"/>
+      <c r="F3" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="36"/>
+      <c r="G3" s="43"/>
+      <c r="H3" s="49"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="33"/>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="34"/>
+      <c r="B4" s="46"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="47"/>
       <c r="F4" s="12" t="s">
         <v>4</v>
       </c>
@@ -2857,22 +3887,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="47" t="s">
+      <c r="A5" s="39" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="48"/>
-      <c r="C5" s="48"/>
-      <c r="D5" s="48"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="48"/>
-      <c r="G5" s="48"/>
-      <c r="H5" s="49"/>
+      <c r="B5" s="40"/>
+      <c r="C5" s="40"/>
+      <c r="D5" s="40"/>
+      <c r="E5" s="40"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="40"/>
+      <c r="H5" s="41"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="28" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="37" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -2895,8 +3925,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="38"/>
-      <c r="B7" s="46"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="38"/>
       <c r="C7" s="20" t="s">
         <v>15</v>
       </c>
@@ -2952,14 +3982,14 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="41"/>
+      <c r="A8" s="31"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="33"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -2997,8 +4027,12 @@
       <c r="AQ8"/>
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="22"/>
-      <c r="B9" s="8"/>
+      <c r="A9" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>36</v>
+      </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
       <c r="E9" s="14"/>
@@ -3469,16 +4503,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="42" t="s">
+      <c r="A19" s="34" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="43"/>
-      <c r="C19" s="43"/>
-      <c r="D19" s="43"/>
-      <c r="E19" s="43"/>
-      <c r="F19" s="43"/>
-      <c r="G19" s="43"/>
-      <c r="H19" s="44"/>
+      <c r="B19" s="35"/>
+      <c r="C19" s="35"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="35"/>
+      <c r="F19" s="35"/>
+      <c r="G19" s="35"/>
+      <c r="H19" s="36"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -3834,16 +4868,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="42" t="s">
+      <c r="A27" s="34" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="43"/>
-      <c r="D27" s="43"/>
-      <c r="E27" s="43"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="43"/>
-      <c r="H27" s="44"/>
+      <c r="B27" s="35"/>
+      <c r="C27" s="35"/>
+      <c r="D27" s="35"/>
+      <c r="E27" s="35"/>
+      <c r="F27" s="35"/>
+      <c r="G27" s="35"/>
+      <c r="H27" s="36"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -3881,8 +4915,12 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="27"/>
-      <c r="B28" s="8"/>
+      <c r="A28" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>40</v>
+      </c>
       <c r="C28" s="15"/>
       <c r="D28" s="15"/>
       <c r="E28" s="15"/>
@@ -4288,6 +5326,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -4295,11 +5338,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -4311,26 +5349,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5c6232be-ce18-4d83-a1a2-d9e20b7892ec">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d67bd3f6-a29a-4795-b867-0d25e089f636" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100829675F584EB7240B97C6F0C1185C021" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="7fbd97b1250289c0d5ac9c8877bdc86d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5c6232be-ce18-4d83-a1a2-d9e20b7892ec" xmlns:ns3="d67bd3f6-a29a-4795-b867-0d25e089f636" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5df9cde456c564a030e5ec79687b571f" ns2:_="" ns3:_="">
     <xsd:import namespace="5c6232be-ce18-4d83-a1a2-d9e20b7892ec"/>
@@ -4537,32 +5555,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2F0E140-9EB4-480C-BE36-83C5DCCA5D99}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="d67bd3f6-a29a-4795-b867-0d25e089f636"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5c6232be-ce18-4d83-a1a2-d9e20b7892ec"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C88069E-52DB-4BCB-B51E-F6679CF16043}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5c6232be-ce18-4d83-a1a2-d9e20b7892ec">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d67bd3f6-a29a-4795-b867-0d25e089f636" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B5A2DA-FF69-471E-A5D4-B38579DF0C44}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -4579,4 +5592,29 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C88069E-52DB-4BCB-B51E-F6679CF16043}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2F0E140-9EB4-480C-BE36-83C5DCCA5D99}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="5c6232be-ce18-4d83-a1a2-d9e20b7892ec"/>
+    <ds:schemaRef ds:uri="d67bd3f6-a29a-4795-b867-0d25e089f636"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Modification tablaeau de synthèse
</commit_message>
<xml_diff>
--- a/Tableau-de-synthèse/8 - BTS SIO - Annexe 8-1 - Tableau de synthèse - Epreuve E4 - BTS SIO 2024.xlsx
+++ b/Tableau-de-synthèse/8 - BTS SIO - Annexe 8-1 - Tableau de synthèse - Epreuve E4 - BTS SIO 2024.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minei\Documents\portfolio_cybersecurite_elegant\Tableau-de-synthèse\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DA94397-9C68-4990-A280-A9477C4C2D94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F9F5279-39E4-4FF2-B791-9A15E4E22683}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,9 +43,6 @@
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="41">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
-  </si>
-  <si>
-    <t>SESSION 2024</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
@@ -182,6 +179,9 @@
   <si>
     <t>05/01/2026 au 20/02/2026</t>
   </si>
+  <si>
+    <t>SESSION 2026</t>
+  </si>
 </sst>
 </file>
 
@@ -750,14 +750,38 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -790,30 +814,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1033,71 +1033,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>512142</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>167130</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>824622</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>438210</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="15" name="Encre 14">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C83C9F4-B448-B837-20A5-6D770290F0EE}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="11864160" y="9090551"/>
-            <a:ext cx="312480" cy="271080"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="15" name="Encre 14">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2C83C9F4-B448-B837-20A5-6D770290F0EE}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="11855520" y="9081551"/>
-              <a:ext cx="330120" cy="288720"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>294620</xdr:colOff>
       <xdr:row>9</xdr:row>
@@ -1111,7 +1046,7 @@
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
       <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId7">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="16" name="Encre 15">
               <a:extLst>
@@ -1228,71 +1163,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>512142</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>178114</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>836142</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>448834</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="23" name="Encre 22">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{285A9A91-08A4-C21A-646B-290C5A44204C}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="11864160" y="9613991"/>
-            <a:ext cx="324000" cy="270720"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="23" name="Encre 22">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{285A9A91-08A4-C21A-646B-290C5A44204C}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId14"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="11855510" y="9605362"/>
-              <a:ext cx="341660" cy="288337"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>608900</xdr:colOff>
       <xdr:row>10</xdr:row>
@@ -1306,7 +1176,7 @@
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
       <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId15">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId13">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="26" name="Encre 25">
               <a:extLst>
@@ -1423,136 +1293,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>490182</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>177938</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>808062</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>416618</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="34" name="Encre 33">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92128C78-56E0-9C55-175D-27D6D2244611}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="11842200" y="10126271"/>
-            <a:ext cx="317880" cy="238680"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="34" name="Encre 33">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{92128C78-56E0-9C55-175D-27D6D2244611}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="11833200" y="10117271"/>
-              <a:ext cx="335520" cy="256320"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>534462</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>211418</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>813102</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>389978</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId21">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="36" name="Encre 35">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B0C1D01-4E31-013B-E14C-43EA25BEA4B7}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="11886480" y="10159751"/>
-            <a:ext cx="278640" cy="178560"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="36" name="Encre 35">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6B0C1D01-4E31-013B-E14C-43EA25BEA4B7}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="11877480" y="10150751"/>
-              <a:ext cx="296280" cy="196200"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>7</xdr:col>
       <xdr:colOff>449420</xdr:colOff>
       <xdr:row>11</xdr:row>
@@ -1566,7 +1306,7 @@
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
       <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId23">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId19">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="39" name="Encre 38">
               <a:extLst>
@@ -1748,71 +1488,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>400182</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>178482</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>880422</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>431202</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="49" name="Encre 48">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75805CF5-3FBC-D1FC-9FF6-EB50D90F4B87}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="11752200" y="10639271"/>
-            <a:ext cx="480240" cy="252720"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="49" name="Encre 48">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{75805CF5-3FBC-D1FC-9FF6-EB50D90F4B87}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="11743200" y="10630271"/>
-              <a:ext cx="497880" cy="270360"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>430284</xdr:colOff>
       <xdr:row>13</xdr:row>
@@ -1826,7 +1501,7 @@
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
       <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId31">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId29">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="50" name="Encre 49">
               <a:extLst>
@@ -1943,71 +1618,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>656862</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>156014</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>980862</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>377414</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
-      <mc:Choice Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35">
-          <xdr14:nvContentPartPr>
-            <xdr14:cNvPr id="55" name="Encre 54">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{536F9B52-94ED-F660-3991-EAFD581D5F47}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr14:cNvPr>
-            <xdr14:cNvContentPartPr/>
-          </xdr14:nvContentPartPr>
-          <xdr14:nvPr macro=""/>
-          <xdr14:xfrm>
-            <a:off x="12008880" y="13925488"/>
-            <a:ext cx="324000" cy="221400"/>
-          </xdr14:xfrm>
-        </xdr:contentPart>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:pic>
-          <xdr:nvPicPr>
-            <xdr:cNvPr id="55" name="Encre 54">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{536F9B52-94ED-F660-3991-EAFD581D5F47}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvPicPr/>
-          </xdr:nvPicPr>
-          <xdr:blipFill>
-            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId36"/>
-            <a:stretch>
-              <a:fillRect/>
-            </a:stretch>
-          </xdr:blipFill>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="11999870" y="13916488"/>
-              <a:ext cx="341660" cy="239040"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-          </xdr:spPr>
-        </xdr:pic>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>282406</xdr:colOff>
       <xdr:row>8</xdr:row>
@@ -2019,9 +1629,9 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>15729</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
-        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId37">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId35">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="4" name="Encre 3">
               <a:extLst>
@@ -2039,7 +1649,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="4" name="Encre 3">
@@ -2084,8 +1694,8 @@
       <xdr:row>8</xdr:row>
       <xdr:rowOff>407945</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId39">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="9" name="Encre 8">
@@ -2104,7 +1714,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="9" name="Encre 8">
@@ -2149,8 +1759,8 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>21863</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId41">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="13" name="Encre 12">
@@ -2169,7 +1779,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="13" name="Encre 12">
@@ -2214,8 +1824,8 @@
       <xdr:row>8</xdr:row>
       <xdr:rowOff>433130</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId43">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="18" name="Encre 17">
@@ -2234,7 +1844,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="18" name="Encre 17">
@@ -2279,8 +1889,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>503083</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId45">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="22" name="Encre 21">
@@ -2299,7 +1909,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="22" name="Encre 21">
@@ -2344,8 +1954,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>424577</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId47">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="27" name="Encre 26">
@@ -2364,7 +1974,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="27" name="Encre 26">
@@ -2409,8 +2019,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>468856</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId49">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="31" name="Encre 30">
@@ -2429,7 +2039,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="31" name="Encre 30">
@@ -2474,8 +2084,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>334620</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId51">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="33" name="Encre 32">
@@ -2494,7 +2104,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="33" name="Encre 32">
@@ -2539,8 +2149,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>412020</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId53">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="37" name="Encre 36">
@@ -2559,7 +2169,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="37" name="Encre 36">
@@ -2604,8 +2214,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>480447</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId55">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="41" name="Encre 40">
@@ -2624,7 +2234,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="41" name="Encre 40">
@@ -2669,8 +2279,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>475864</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing">
+      <mc:Choice Requires="xdr14">
         <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId57">
           <xdr14:nvContentPartPr>
             <xdr14:cNvPr id="46" name="Encre 45">
@@ -2689,7 +2299,7 @@
           </xdr14:xfrm>
         </xdr:contentPart>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:pic>
           <xdr:nvPicPr>
             <xdr:cNvPr id="46" name="Encre 45">
@@ -2711,6 +2321,266 @@
             <a:xfrm>
               <a:off x="14384160" y="17715478"/>
               <a:ext cx="486000" cy="359640"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>423305</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>167045</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>935945</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>323285</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId59">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="3" name="Encre 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{127EB3A9-4BA9-7595-1034-214D31586486}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="9168480" y="13936519"/>
+            <a:ext cx="512640" cy="156240"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="3" name="Encre 2">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{127EB3A9-4BA9-7595-1034-214D31586486}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId60"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="9159840" y="13927519"/>
+              <a:ext cx="530280" cy="173880"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>456425</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>78125</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>827945</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>365045</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId61">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="5" name="Encre 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D45EF160-103A-B7AA-CADF-AF0E911A6658}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="9201600" y="13847599"/>
+            <a:ext cx="371520" cy="286920"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="5" name="Encre 4">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D45EF160-103A-B7AA-CADF-AF0E911A6658}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId62"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="9192600" y="13838599"/>
+              <a:ext cx="389160" cy="304560"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>256404</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>133186</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>857964</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>465106</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId63">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="12" name="Encre 11">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED06FE35-4B35-E2D9-22AC-00F6996F6484}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="10305000" y="13902660"/>
+            <a:ext cx="601560" cy="331920"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="12" name="Encre 11">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ED06FE35-4B35-E2D9-22AC-00F6996F6484}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId64"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="10296000" y="13894020"/>
+              <a:ext cx="619200" cy="349560"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+          </xdr:spPr>
+        </xdr:pic>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>253801</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>133836</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>957961</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>422916</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" Requires="xdr14">
+        <xdr:contentPart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId65">
+          <xdr14:nvContentPartPr>
+            <xdr14:cNvPr id="20" name="Encre 19">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C53DB5B-BC34-7E78-48E6-73EF38004D83}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr14:cNvPr>
+            <xdr14:cNvContentPartPr/>
+          </xdr14:nvContentPartPr>
+          <xdr14:nvPr macro=""/>
+          <xdr14:xfrm>
+            <a:off x="12909240" y="9569713"/>
+            <a:ext cx="704160" cy="289080"/>
+          </xdr14:xfrm>
+        </xdr:contentPart>
+      </mc:Choice>
+      <mc:Fallback>
+        <xdr:pic>
+          <xdr:nvPicPr>
+            <xdr:cNvPr id="20" name="Encre 19">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5C53DB5B-BC34-7E78-48E6-73EF38004D83}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvPicPr/>
+          </xdr:nvPicPr>
+          <xdr:blipFill>
+            <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId66"/>
+            <a:stretch>
+              <a:fillRect/>
+            </a:stretch>
+          </xdr:blipFill>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="12900240" y="9560713"/>
+              <a:ext cx="721800" cy="306720"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -2767,115 +2637,6 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:06:48.688"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 0 24575,'98'50'0,"97"51"0,-174-89 0,-2 0 0,0 2 0,0 0 0,-1 1 0,-1 0 0,0 2 0,19 24 0,66 72 0,-18-22 0,-72-78 0,1-1 0,0 0 0,1-1 0,0-1 0,0 0 0,17 7 0,8 7 0,33 23-1365,-57-36-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink11.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:06:51.272"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">773 0 24097,'-773'495'0</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink12.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:06:59.489"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1290 0 24575,'-27'11'0,"-34"19"0,-44 20 0,-42 18 0,-10 7 0,4 2-1061,9-7 1061,17-16 0,31-11 260,26-8-260,20-10 0,13-9 0,7-7 0,10 0 0,2-2 801,-1-2-801,3 4 0,4 0-8191</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1233.49">83 32 24575,'33'13'0,"0"1"0,-1 1 0,-1 2 0,44 31 0,105 95 0,-127-98 0,173 154 0,-163-152 307,-46-35-725,0 0 0,-1 1 0,23 24 0,-28-24-6408</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink13.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:07:17.204"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1354 0 24575,'-52'3'0,"-100"17"0,135-17 0,-85 19 0,-147 52 0,170-47 0,-14 9 0,21-6 0,-77 40 0,46-19 0,-16-9 333,77-28-1182,-58 26 0,75-26-5977</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink14.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:07:18.641"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -2887,35 +2648,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink15.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:07:22.391"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1333 0 24575,'-9'1'0,"1"1"0,0-1 0,0 1 0,0 1 0,0 0 0,0 0 0,0 1 0,1-1 0,-11 9 0,-10 3 0,-322 145 0,123-52 0,-71 29 0,-17-20-1365,290-109-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1449.1">157 216 24575,'5'0'0,"-1"1"0,1 0 0,-1 0 0,0 0 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 1 0,6 3 0,6 4 0,66 35 0,-2 4 0,-2 4 0,95 83 0,-130-96 0,-18-16 0,44 33 0,-12-16-1365,-41-31-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink11.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -2942,7 +2675,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink12.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -2969,35 +2702,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink18.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:08:07.087"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">899 0 24575,'-18'2'0,"0"0"0,0 2 0,1 0 0,-1 0 0,1 2 0,0 0 0,0 1 0,-16 10 0,-14 11 0,36-19 0,-2-2 0,1 0 0,-21 9 0,19-10 0,1 0 0,0 0 0,1 2 0,-1-1 0,-15 14 0,-53 54 0,32-28 0,13-16 0,-1-2 0,-1-1 0,-46 24 0,74-46 35,-82 51-1435,78-47-5426</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1588.16">0 155 24575,'242'120'0,"-222"-107"0,0 1 0,0 0 0,-2 1 0,0 1 0,29 33 0,-39-41 0,0-1 0,1 0 0,0 0 0,12 6 0,22 16 0,25 24 0,-39-32 0,35 33 0,-63-53 1,-1-1-48,1 0 0,-1 1 0,1-1 0,0 1-1,-1-1 1,1 1 0,-1-1 0,1 1 0,-1-1 0,0 1 0,1-1 0,-1 1 0,0 0 0,1-1-1,-1 1 1,0 0 0,0-1 0,1 1 0,-1 0 0,0-1 0,0 1 0,0 0 0,0-1-1,0 1 1,0 0 0,0 0 0,0-1 0,0 2 0</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink13.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -3022,6 +2727,174 @@
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">1969 216 24575,'-360'111'-289,"10"21"-291,267-100 446,-743 312 121,595-244 164,211-92-276,2 0 0,-1 2 0,-30 21 0,36-20-6701</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1613.33">422 0 24575,'23'1'0,"0"1"0,0 2 0,38 9 0,-43-9 0,482 162 0,-392-126 0,-5 1 0,-41-16 0,75 20 0,-123-41 0,-1 1 0,0 0 0,0 1 0,-1 0 0,21 13 0,-6 1 0,29 27 0,1-5 0,-40-31 0,27 23 0,17 27 0,-33-32 0,2-1 0,47 35 0,16-9-1365,-70-42-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink14.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:14:26.544"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1540 278 24575,'-31'5'0,"-48"13"0,-42 13 0,-37 18 0,-18 11-1438,-5 5 1438,7-2 0,11-8 0,24-7 0,30-12 0,28-7 468,23-8-468,16-8 238,15-5-7697</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2213.43">86 1 24575,'10'0'0,"0"2"0,1-1 0,-1 1 0,0 1 0,0 0 0,0 0 0,-1 1 0,17 8 0,72 50 0,-76-47 0,88 66 0,-65-46 0,1-2 0,55 31 0,-76-50 0,36 28 0,-42-27 0,0-1 0,43 21 0,7 0 0,76 52 0,-134-79 0,0 0 0,13 14 0,-17-15 0,1 0 0,1 0 0,-1 0 0,17 9 0,-16-12 0,11 6 0,0 0 0,0 2 0,25 20 0,-21-11 110,-8-6-479,1-1 1,0 0-1,37 22 0,-32-25-6457</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink15.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:15:07.744"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1732 373 24575,'-26'1'0,"-1"1"0,2 1 0,-1 1 0,-29 9 0,-98 39 0,123-41 0,-734 334 0,420-166 0,266-136 231,49-26-630,0-2 0,-1 0 0,-59 19 0,63-28-6427</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1432.1">246 1 24575,'4'0'0,"1"0"0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,1 0 0,4 4 0,5 5 0,22 20 0,-4-3 0,70 41 0,-62-43 0,52 43 0,94 94 0,-121-106 0,36 28 0,-53-55 0,-33-21 0,-1 0 0,0 1 0,-1 0 0,19 18 0,-7 0 0,-14-15 0,0-1 0,1 0 0,0-1 0,19 14 0,60 44 0,-60-43 0,49 30 0,-39-39 312,-12-6-1989,-12-2-5149</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink16.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:15:26.188"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1547 31 24575,'-31'10'0,"-43"15"0,-45 29 0,-39 15 0,-19 2-1835,-6 5 1835,17-1 0,22-7 0,19-10 0,26-16 593,19-8-593,18-11 303,14-4-303,11-5 0,10 0 0,11-2-7252</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1451.2">0 1 24575,'49'26'0,"59"44"0,-64-41 0,198 149 0,-149-108 0,189 161 0,-264-215 0,5 1-227,-1 0-1,2-1 1,0-1-1,1-2 1,44 18-1,-43-22-6598</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink17.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:19:13.265"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1422 125 24575,'-5'0'0,"1"0"0,-1 1 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-6 4 0,-10 3 0,-727 309 0,551-228 0,112-59 0,56-21 0,-45 21 0,3 4 0,-38 20 0,84-40-1365,2-3-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1166.08">153 1 24575,'23'9'0,"0"1"0,31 18 0,-16-7 0,609 364 0,-45 34 0,-305-193-1365,-272-205-5461</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink18.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:09.892"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1873 247 24575,'-40'9'0,"0"1"0,1 2 0,-38 18 0,42-16 0,-506 206-650,-293 107-576,595-236 2524,236-90-1256,1 0-1,-1 0 1,1 0 0,-1 0 0,1 0-1,-1 1 1,1-1 0,-4 4 0,6-5-38,0 1 0,0-1 1,0 0-1,0 0 0,-1 0 0,1 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 1-1,-1-1 0,1 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,1 1-1,-1-1 0,0 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 0-1,0 1 0,1-1 0,14 6 54,35-2-1423,-23-3-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1863.49">325 0 24575,'8'1'0,"-2"-1"0,1 1 0,0 1 0,0-1 0,0 1 0,0 1 0,-1-1 0,1 1 0,-1 0 0,7 5 0,8 6 0,28 23 0,-45-34 0,188 132 0,-40-33 0,-44-34 0,-70-47 0,37 28 0,152 125 0,-218-167 0,0 0 0,0 1 0,-1 0 0,0 0 0,0 1 0,6 10 0,-10-14 0,-1 0 0,1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,7 4 0,49 22 0,-48-25 0,0 1 0,0 1 0,0 0 0,17 13 0,-6-1-6,48 28-1,-39-27-1345,-17-9-5474</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink19.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:21.810"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">2078 62 24575,'-51'1'0,"0"3"0,0 2 0,-67 17 0,-143 54 0,131-36 0,-366 99 0,391-113 0,59-16 0,-70 25 0,19-1 0,58-23 0,2 2 0,-68 36 0,79-37 0,0-1 0,-51 17 0,-17 6 0,49-15 0,-46 23 0,90-42 25,-1-1-1,1 1 0,0-1 1,0 1-1,0 0 1,0 0-1,0 0 0,0 0 1,0-1-1,0 1 0,0 0 1,0 1-1,-1 0 1,3-2-77,-1 1 0,0-1 0,0 1 1,1-1-1,-1 1 0,0-1 1,0 1-1,1-1 0,-1 0 0,1 1 1,-1-1-1,0 0 0,1 1 1,-1-1-1,1 0 0,-1 1 0,0-1 1,1 0-1,-1 0 0,1 0 1,-1 1-1,1-1 0,-1 0 0,1 0 1,-1 0-1,1 0 0,-1 0 1,1 0-1,-1 0 0,1 0 0,-1 0 1,2 0-1,19 2-6774</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1234.68">437 0 24575,'487'193'-835,"-28"46"100,-233-103 985,-179-103 121,-1 1 0,63 64 1,-100-90-281,0 0 1,16 10 0,-18-15-251,-1 1-1,0 1 1,0-1 0,-1 1-1,1 0 1,-1 0 0,0 1-1,8 11 1,-6-1-6667</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -3068,174 +2941,6 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:14:26.544"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1540 278 24575,'-31'5'0,"-48"13"0,-42 13 0,-37 18 0,-18 11-1438,-5 5 1438,7-2 0,11-8 0,24-7 0,30-12 0,28-7 468,23-8-468,16-8 238,15-5-7697</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="2213.43">86 1 24575,'10'0'0,"0"2"0,1-1 0,-1 1 0,0 1 0,0 0 0,0 0 0,-1 1 0,17 8 0,72 50 0,-76-47 0,88 66 0,-65-46 0,1-2 0,55 31 0,-76-50 0,36 28 0,-42-27 0,0-1 0,43 21 0,7 0 0,76 52 0,-134-79 0,0 0 0,13 14 0,-17-15 0,1 0 0,1 0 0,-1 0 0,17 9 0,-16-12 0,11 6 0,0 0 0,0 2 0,25 20 0,-21-11 110,-8-6-479,1-1 1,0 0-1,37 22 0,-32-25-6457</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink21.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:15:07.744"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1732 373 24575,'-26'1'0,"-1"1"0,2 1 0,-1 1 0,-29 9 0,-98 39 0,123-41 0,-734 334 0,420-166 0,266-136 231,49-26-630,0-2 0,-1 0 0,-59 19 0,63-28-6427</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1432.1">246 1 24575,'4'0'0,"1"0"0,0 1 0,-1 0 0,1 0 0,-1 0 0,1 1 0,-1-1 0,0 1 0,0 0 0,1 0 0,4 4 0,5 5 0,22 20 0,-4-3 0,70 41 0,-62-43 0,52 43 0,94 94 0,-121-106 0,36 28 0,-53-55 0,-33-21 0,-1 0 0,0 1 0,-1 0 0,19 18 0,-7 0 0,-14-15 0,0-1 0,1 0 0,0-1 0,19 14 0,60 44 0,-60-43 0,49 30 0,-39-39 312,-12-6-1989,-12-2-5149</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink22.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:15:26.188"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1547 31 24575,'-31'10'0,"-43"15"0,-45 29 0,-39 15 0,-19 2-1835,-6 5 1835,17-1 0,22-7 0,19-10 0,26-16 593,19-8-593,18-11 303,14-4-303,11-5 0,10 0 0,11-2-7252</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1451.2">0 1 24575,'49'26'0,"59"44"0,-64-41 0,198 149 0,-149-108 0,189 161 0,-264-215 0,5 1-227,-1 0-1,2-1 1,0-1-1,1-2 1,44 18-1,-43-22-6598</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink23.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:19:13.265"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1422 125 24575,'-5'0'0,"1"0"0,-1 1 0,1-1 0,0 1 0,-1 0 0,1 0 0,0 0 0,0 0 0,-6 4 0,-10 3 0,-727 309 0,551-228 0,112-59 0,56-21 0,-45 21 0,3 4 0,-38 20 0,84-40-1365,2-3-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1166.09">153 1 24575,'23'9'0,"0"1"0,31 18 0,-16-7 0,609 364 0,-45 34 0,-305-193-1365,-272-205-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink24.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:09.892"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">1873 247 24575,'-40'9'0,"0"1"0,1 2 0,-38 18 0,42-16 0,-506 206-650,-293 107-576,595-236 2524,236-90-1256,1 0-1,-1 0 1,1 0 0,-1 0 0,1 0-1,-1 1 1,1-1 0,-4 4 0,6-5-38,0 1 0,0-1 1,0 0-1,0 0 0,-1 0 0,1 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 1-1,-1-1 0,1 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,1 1-1,-1-1 0,0 0 0,0 0 1,0 1-1,0-1 0,0 0 0,0 0 1,0 0-1,0 1 0,1-1 0,14 6 54,35-2-1423,-23-3-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1863.49">325 0 24575,'8'1'0,"-2"-1"0,1 1 0,0 1 0,0-1 0,0 1 0,0 1 0,-1-1 0,1 1 0,-1 0 0,7 5 0,8 6 0,28 23 0,-45-34 0,188 132 0,-40-33 0,-44-34 0,-70-47 0,37 28 0,152 125 0,-218-167 0,0 0 0,0 1 0,-1 0 0,0 0 0,0 1 0,6 10 0,-10-14 0,-1 0 0,1-1 0,1 1 0,-1-1 0,1 0 0,-1 0 0,1 0 0,7 4 0,49 22 0,-48-25 0,0 1 0,0 1 0,0 0 0,17 13 0,-6-1-6,48 28-1,-39-27-1345,-17-9-5474</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink25.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:21.810"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">2078 62 24575,'-51'1'0,"0"3"0,0 2 0,-67 17 0,-143 54 0,131-36 0,-366 99 0,391-113 0,59-16 0,-70 25 0,19-1 0,58-23 0,2 2 0,-68 36 0,79-37 0,0-1 0,-51 17 0,-17 6 0,49-15 0,-46 23 0,90-42 25,-1-1-1,1 1 0,0-1 1,0 1-1,0 0 1,0 0-1,0 0 0,0 0 1,0-1-1,0 1 0,0 0 1,0 1-1,-1 0 1,3-2-77,-1 1 0,0-1 0,0 1 1,1-1-1,-1 1 0,0-1 1,0 1-1,1-1 0,-1 0 0,1 1 1,-1-1-1,0 0 0,1 1 1,-1-1-1,1 0 0,-1 1 0,0-1 1,1 0-1,-1 0 0,1 0 1,-1 1-1,1-1 0,-1 0 0,1 0 1,-1 0-1,1 0 0,-1 0 1,1 0-1,-1 0 0,1 0 0,-1 0 1,2 0-1,19 2-6774</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1234.69">437 0 24575,'487'193'-835,"-28"46"100,-233-103 985,-179-103 121,-1 1 0,63 64 1,-100-90-281,0 0 1,16 10 0,-18-15-251,-1 1-1,0 1 1,0-1 0,-1 1-1,1 0 1,-1 0 0,0 1-1,8 11 1,-6-1-6667</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink26.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2026-03-21T18:20:32.915"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -3247,7 +2952,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink21.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -3274,7 +2979,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink28.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink22.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -3302,7 +3007,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink29.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink23.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -3327,6 +3032,116 @@
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">1300 62 24575,'-2'0'0,"0"0"0,0 0 0,0 1 0,-1-1 0,1 1 0,0-1 0,0 1 0,0 0 0,0 0 0,0 0 0,-3 2 0,-9 5 0,-411 156 0,21-10 0,299-116 0,78-29 0,0 0 0,0 1 0,1 2 0,-25 15 0,-54 35-1365,80-50-5461</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1460.05">0 0 24575,'1'3'0,"0"0"0,1-1 0,-1 1 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 0 0,0 1 0,0-1 0,4 3 0,2 5 0,16 15 0,1 0 0,1-2 0,50 36 0,-50-40 0,-6-1 0,0 1 0,-1 0 0,-1 1 0,25 38 0,7 7 0,31 29 0,110 100 0,-156-159 167,36 47 0,-46-51-734,2-1 1,51 45 0,-59-60-6260</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink24.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-28T07:48:28.624"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1423 0 24093,'-1422'433'0</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink25.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-28T07:48:30.051"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">0 0 24575,'19'1'0,"0"0"0,0 2 0,0 0 0,0 1 0,0 1 0,-1 1 0,32 14 0,-13-1 0,-1 1 0,53 39 0,-69-43 0,-1 1 0,-1 1 0,18 22 0,1 1 0,-8-5 0,-21-25 0,1-1 0,17 17 0,-15-15 0,1 0 0,-2 0 0,18 27 0,-17-22 0,25 27 0,111 90 0,-103-96 0,-12-11-341,0-1 0,1-2-1,38 21 1,-53-36-6485</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink26.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-28T07:49:03.999"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1670 125 24575,'-37'3'0,"0"0"0,-46 12 0,34-6 0,-371 88 0,282-62 0,94-26 0,-66 5 0,25-4 0,-100 32 0,169-38 0,-163 52 0,169-53 0,-71 28 0,-23 6 0,55-20-1365,29-9-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1320.88">0 1 24575,'5'4'0,"0"0"0,0 0 0,0 0 0,1 0 0,-1-1 0,8 3 0,4 3 0,69 39 0,280 173 0,-111-51 0,90 65 0,-311-207 165,50 52 1,8 8-1862,-75-75-5130</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink27.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2026-03-28T07:57:44.155"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1956 93 24575,'-13'1'0,"1"0"0,0 1 0,0 0 0,-1 0 0,1 2 0,-15 5 0,-68 36 0,56-26 0,-562 249 0,485-219 0,-145 52 0,-412 89 0,634-181-1365,9-2-5461</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1938.72">317 0 24575,'19'1'0,"-1"0"0,1 2 0,-1 0 0,19 6 0,70 26 0,-83-26 0,356 149 0,-204-59 0,-27-15 0,-42-16 0,-74-45 0,57 30 0,-72-44 0,0 1 0,-1 2 0,-1-1 0,0 2 0,25 24 0,-21-19 86,0-1-1,2-1 0,28 16 1,72 33-1793,-105-56-5119</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -3375,34 +3190,6 @@
           <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
         </inkml:channelProperties>
       </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:05:41.076"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">867 155 24575,'-6'0'0,"-1"0"0,1 1 0,-1 0 0,1 1 0,0-1 0,-1 1 0,1 1 0,-9 4 0,-43 29 0,46-29 0,-43 32 0,-204 125 0,141-94 0,42-23 0,29-26 0,36-17 0,0 0 0,-17 11 0,18-9-273,-1 0 0,0 0 0,0-1 0,-16 5 0,5-4-6553</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1293.32">1 0 24575,'0'3'0,"1"0"0,0 0 0,1 0 0,-1 0 0,0 0 0,1-1 0,-1 1 0,1-1 0,0 1 0,0-1 0,0 1 0,0-1 0,0 0 0,4 3 0,3 4 0,132 127 0,-80-79 0,60 71 0,-75-75 0,52 48 0,-35-32 0,-32-32 0,61 67-1365,-80-88-5461</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink5.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
       <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:05:44.108"/>
     </inkml:context>
     <inkml:brush xml:id="br0">
@@ -3414,7 +3201,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink5.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -3441,35 +3228,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink7.xml><?xml version="1.0" encoding="utf-8"?>
-<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
-  <inkml:definitions>
-    <inkml:context xml:id="ctx0">
-      <inkml:inkSource xml:id="inkSrc0">
-        <inkml:traceFormat>
-          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
-          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
-        </inkml:traceFormat>
-        <inkml:channelProperties>
-          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
-          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
-        </inkml:channelProperties>
-      </inkml:inkSource>
-      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:06:03.079"/>
-    </inkml:context>
-    <inkml:brush xml:id="br0">
-      <inkml:brushProperty name="width" value="0.05" units="cm"/>
-      <inkml:brushProperty name="height" value="0.05" units="cm"/>
-    </inkml:brush>
-  </inkml:definitions>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0">899 1 24575,'-2'2'0,"-1"0"0,1 0 0,-1 0 0,1 0 0,-1-1 0,1 1 0,-5 1 0,-11 7 0,-135 96 0,37-24 0,85-61 0,-194 121 0,191-121 0,-45 35 0,56-38 0,0-1 0,-1-1 0,0-1 0,-36 15 0,32-18-1365,7-1-5461</inkml:trace>
-  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1212.23">1 155 24575,'4'1'0,"-1"0"0,1 0 0,0 1 0,0-1 0,-1 1 0,1 0 0,-1 0 0,0 0 0,1 0 0,4 5 0,4 2 0,248 170 0,-12 21 0,-183-144 253,-36-32-792,0 1-1,36 42 1,-54-53-6287</inkml:trace>
-</inkml:ink>
-</file>
-
-<file path=xl/ink/ink8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink6.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -3497,7 +3256,7 @@
 </inkml:ink>
 </file>
 
-<file path=xl/ink/ink9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/ink/ink7.xml><?xml version="1.0" encoding="utf-8"?>
 <inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
   <inkml:definitions>
     <inkml:context xml:id="ctx0">
@@ -3522,6 +3281,61 @@
   </inkml:definitions>
   <inkml:trace contextRef="#ctx0" brushRef="#br0">1014 61 24575,'-21'6'0,"-29"11"0,-31 20 0,-23 13 0,-21 9 0,1 0 0,6-5 0,17-1 0,16-10 0,16-7 0,16-9 0,16-4 0,9-6 0,10-6-8191</inkml:trace>
   <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1286.05">115 0 24575,'3'1'0,"0"0"0,0 0 0,0 0 0,-1 1 0,1-1 0,-1 1 0,1 0 0,-1-1 0,0 1 0,1 0 0,2 4 0,4 3 0,69 45 0,9 8 0,20 40 0,-83-80 0,-2 0 0,31 41 0,-33-38 0,1 0 0,33 29 0,-40-42-227,-1 2-1,-1-1 1,0 2-1,0 0 1,17 31-1,-19-27-6598</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink8.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:06:59.489"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1290 0 24575,'-27'11'0,"-34"19"0,-44 20 0,-42 18 0,-10 7 0,4 2-1061,9-7 1061,17-16 0,31-11 260,26-8-260,20-10 0,13-9 0,7-7 0,10 0 0,2-2 801,-1-2-801,3 4 0,4 0-8191</inkml:trace>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0" timeOffset="1233.49">83 32 24575,'33'13'0,"0"1"0,-1 1 0,-1 2 0,44 31 0,105 95 0,-127-98 0,173 154 0,-163-152 307,-46-35-725,0 0 0,-1 1 0,23 24 0,-28-24-6408</inkml:trace>
+</inkml:ink>
+</file>
+
+<file path=xl/ink/ink9.xml><?xml version="1.0" encoding="utf-8"?>
+<inkml:ink xmlns:inkml="http://www.w3.org/2003/InkML">
+  <inkml:definitions>
+    <inkml:context xml:id="ctx0">
+      <inkml:inkSource xml:id="inkSrc0">
+        <inkml:traceFormat>
+          <inkml:channel name="X" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="Y" type="integer" min="-2.14748E9" max="2.14748E9" units="cm"/>
+          <inkml:channel name="F" type="integer" max="32767" units="dev"/>
+        </inkml:traceFormat>
+        <inkml:channelProperties>
+          <inkml:channelProperty channel="X" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="Y" name="resolution" value="1000" units="1/cm"/>
+          <inkml:channelProperty channel="F" name="resolution" value="0" units="1/dev"/>
+        </inkml:channelProperties>
+      </inkml:inkSource>
+      <inkml:timestamp xml:id="ts0" timeString="2025-12-14T20:07:17.204"/>
+    </inkml:context>
+    <inkml:brush xml:id="br0">
+      <inkml:brushProperty name="width" value="0.05" units="cm"/>
+      <inkml:brushProperty name="height" value="0.05" units="cm"/>
+    </inkml:brush>
+  </inkml:definitions>
+  <inkml:trace contextRef="#ctx0" brushRef="#br0">1354 0 24575,'-52'3'0,"-100"17"0,135-17 0,-85 19 0,-147 52 0,170-47 0,-14 9 0,21-6 0,-77 40 0,46-19 0,-16-9 333,77-28-1182,-58 26 0,75-26-5977</inkml:trace>
 </inkml:ink>
 </file>
 
@@ -3826,124 +3640,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-      <c r="D1" s="30"/>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="30" t="s">
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28" t="s">
+        <v>40</v>
+      </c>
+      <c r="H1" s="28"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="28" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="30"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="30"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="28"/>
+      <c r="G2" s="28"/>
+      <c r="H2" s="28"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="42" t="s">
-        <v>24</v>
+      <c r="A3" s="29" t="s">
+        <v>23</v>
       </c>
-      <c r="B3" s="43"/>
-      <c r="C3" s="43"/>
-      <c r="D3" s="43"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="48" t="s">
-        <v>37</v>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="35" t="s">
+        <v>36</v>
       </c>
-      <c r="G3" s="43"/>
-      <c r="H3" s="49"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="36"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="32" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="33"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="34"/>
+      <c r="F4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="46"/>
-      <c r="D4" s="46"/>
-      <c r="E4" s="47"/>
-      <c r="F4" s="12" t="s">
+      <c r="G4" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="13" t="s">
+      <c r="H4" s="19" t="s">
         <v>5</v>
-      </c>
-      <c r="H4" s="19" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="39" t="s">
-        <v>25</v>
+      <c r="A5" s="47" t="s">
+        <v>24</v>
       </c>
-      <c r="B5" s="40"/>
-      <c r="C5" s="40"/>
-      <c r="D5" s="40"/>
-      <c r="E5" s="40"/>
-      <c r="F5" s="40"/>
-      <c r="G5" s="40"/>
-      <c r="H5" s="41"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="48"/>
+      <c r="D5" s="48"/>
+      <c r="E5" s="48"/>
+      <c r="F5" s="48"/>
+      <c r="G5" s="48"/>
+      <c r="H5" s="49"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="37" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="45" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="37" t="s">
+      <c r="C6" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="D6" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="7" t="s">
         <v>13</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="29"/>
-      <c r="B7" s="38"/>
+      <c r="A7" s="38"/>
+      <c r="B7" s="46"/>
       <c r="C7" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="E7" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="20" t="s">
+      <c r="F7" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="20" t="s">
+      <c r="G7" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="G7" s="20" t="s">
+      <c r="H7" s="21" t="s">
         <v>19</v>
-      </c>
-      <c r="H7" s="21" t="s">
-        <v>20</v>
       </c>
       <c r="I7"/>
       <c r="J7"/>
@@ -3982,14 +3796,14 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="31"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="33"/>
+      <c r="A8" s="39"/>
+      <c r="B8" s="40"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
+      <c r="H8" s="41"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -4028,10 +3842,10 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="22" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -4077,10 +3891,10 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="14"/>
       <c r="D10" s="14"/>
@@ -4126,10 +3940,10 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11" s="25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C11" s="14"/>
       <c r="D11" s="14"/>
@@ -4175,10 +3989,10 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="14"/>
       <c r="D12" s="14"/>
@@ -4193,7 +4007,7 @@
       <c r="M12"/>
       <c r="N12"/>
       <c r="O12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="P12"/>
       <c r="Q12"/>
@@ -4226,10 +4040,10 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="26" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" s="15"/>
       <c r="D13" s="15"/>
@@ -4275,10 +4089,10 @@
     </row>
     <row r="14" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="26" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14" s="15"/>
       <c r="D14" s="15"/>
@@ -4503,16 +4317,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="34" t="s">
-        <v>22</v>
+      <c r="A19" s="42" t="s">
+        <v>21</v>
       </c>
-      <c r="B19" s="35"/>
-      <c r="C19" s="35"/>
-      <c r="D19" s="35"/>
-      <c r="E19" s="35"/>
-      <c r="F19" s="35"/>
-      <c r="G19" s="35"/>
-      <c r="H19" s="36"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="43"/>
+      <c r="D19" s="43"/>
+      <c r="E19" s="43"/>
+      <c r="F19" s="43"/>
+      <c r="G19" s="43"/>
+      <c r="H19" s="44"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -4551,10 +4365,10 @@
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="27" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B20" s="25" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20" s="15"/>
       <c r="D20" s="15"/>
@@ -4868,16 +4682,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="34" t="s">
-        <v>23</v>
+      <c r="A27" s="42" t="s">
+        <v>22</v>
       </c>
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
-      <c r="H27" s="36"/>
+      <c r="B27" s="43"/>
+      <c r="C27" s="43"/>
+      <c r="D27" s="43"/>
+      <c r="E27" s="43"/>
+      <c r="F27" s="43"/>
+      <c r="G27" s="43"/>
+      <c r="H27" s="44"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -4916,10 +4730,10 @@
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C28" s="15"/>
       <c r="D28" s="15"/>
@@ -5326,11 +5140,6 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -5338,6 +5147,11 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -5349,6 +5163,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5c6232be-ce18-4d83-a1a2-d9e20b7892ec">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d67bd3f6-a29a-4795-b867-0d25e089f636" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100829675F584EB7240B97C6F0C1185C021" ma:contentTypeVersion="13" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="7fbd97b1250289c0d5ac9c8877bdc86d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5c6232be-ce18-4d83-a1a2-d9e20b7892ec" xmlns:ns3="d67bd3f6-a29a-4795-b867-0d25e089f636" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5df9cde456c564a030e5ec79687b571f" ns2:_="" ns3:_="">
     <xsd:import namespace="5c6232be-ce18-4d83-a1a2-d9e20b7892ec"/>
@@ -5555,27 +5389,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2F0E140-9EB4-480C-BE36-83C5DCCA5D99}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="5c6232be-ce18-4d83-a1a2-d9e20b7892ec"/>
+    <ds:schemaRef ds:uri="d67bd3f6-a29a-4795-b867-0d25e089f636"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5c6232be-ce18-4d83-a1a2-d9e20b7892ec">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d67bd3f6-a29a-4795-b867-0d25e089f636" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C88069E-52DB-4BCB-B51E-F6679CF16043}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A7B5A2DA-FF69-471E-A5D4-B38579DF0C44}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5592,29 +5431,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8C88069E-52DB-4BCB-B51E-F6679CF16043}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2F0E140-9EB4-480C-BE36-83C5DCCA5D99}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="5c6232be-ce18-4d83-a1a2-d9e20b7892ec"/>
-    <ds:schemaRef ds:uri="d67bd3f6-a29a-4795-b867-0d25e089f636"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>